<commit_message>
feat: add admin code validation and watermark option for PDF generation
</commit_message>
<xml_diff>
--- a/public/exampleExcel.xlsx
+++ b/public/exampleExcel.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29530"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29725"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/aba03c58143b1879/Documentos/Repositorios/generator_id_card/public/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{FC7CF8CC-3A12-4D65-83A3-A2446F137DD2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="6" documentId="8_{FC7CF8CC-3A12-4D65-83A3-A2446F137DD2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{13C99C88-36B1-4EA7-9B16-4FC3B75B00C5}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{63B3DDDE-9EB7-4985-ADA3-F3ED766A51FF}"/>
   </bookViews>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="11" uniqueCount="11">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="15" uniqueCount="15">
   <si>
     <t>nombres</t>
   </si>
@@ -69,6 +69,18 @@
   </si>
   <si>
     <t>Sexto</t>
+  </si>
+  <si>
+    <t>Test 1</t>
+  </si>
+  <si>
+    <t>test 2</t>
+  </si>
+  <si>
+    <t>Septimo</t>
+  </si>
+  <si>
+    <t>Once</t>
   </si>
 </sst>
 </file>
@@ -440,7 +452,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{28AF2DEA-5356-4DA3-BE68-E5CEC210EB8D}">
-  <dimension ref="A1:C5"/>
+  <dimension ref="A1:C7"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <sheetData>
     <row r="1" spans="1:3" x14ac:dyDescent="0.25">
@@ -498,6 +510,28 @@
         <v>1024528857</v>
       </c>
     </row>
+    <row r="6" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A6" t="s">
+        <v>11</v>
+      </c>
+      <c r="B6" t="s">
+        <v>13</v>
+      </c>
+      <c r="C6">
+        <v>123456789</v>
+      </c>
+    </row>
+    <row r="7" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A7" t="s">
+        <v>12</v>
+      </c>
+      <c r="B7" t="s">
+        <v>14</v>
+      </c>
+      <c r="C7">
+        <v>321654897</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>

<commit_message>
feat: add admin code validation and watermark logic for PDF generation
</commit_message>
<xml_diff>
--- a/public/exampleExcel.xlsx
+++ b/public/exampleExcel.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/aba03c58143b1879/Documentos/Repositorios/generator_id_card/public/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="6" documentId="8_{FC7CF8CC-3A12-4D65-83A3-A2446F137DD2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{13C99C88-36B1-4EA7-9B16-4FC3B75B00C5}"/>
+  <xr:revisionPtr revIDLastSave="10" documentId="8_{FC7CF8CC-3A12-4D65-83A3-A2446F137DD2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{16225422-DECD-40EE-8B0D-93D45C9B6F1F}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{63B3DDDE-9EB7-4985-ADA3-F3ED766A51FF}"/>
   </bookViews>
@@ -74,13 +74,13 @@
     <t>Test 1</t>
   </si>
   <si>
+    <t>Septimo</t>
+  </si>
+  <si>
     <t>test 2</t>
   </si>
   <si>
-    <t>Septimo</t>
-  </si>
-  <si>
-    <t>Once</t>
+    <t>once</t>
   </si>
 </sst>
 </file>
@@ -133,6 +133,10 @@
     </ext>
   </extLst>
 </styleSheet>
+</file>
+
+<file path=xl/persons/person.xml><?xml version="1.0" encoding="utf-8"?>
+<personList xmlns="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main"/>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -515,7 +519,7 @@
         <v>11</v>
       </c>
       <c r="B6" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="C6">
         <v>123456789</v>
@@ -523,13 +527,13 @@
     </row>
     <row r="7" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="B7" t="s">
         <v>14</v>
       </c>
       <c r="C7">
-        <v>321654897</v>
+        <v>9865423185</v>
       </c>
     </row>
   </sheetData>

</xml_diff>